<commit_message>
Update reference file: Y4_B2526_General_&_Special_Surgery_1_A2_reference_data.xlsx
</commit_message>
<xml_diff>
--- a/reference_data/Y4_B2526_General_&_Special_Surgery_1_A2_reference_data.xlsx
+++ b/reference_data/Y4_B2526_General_&_Special_Surgery_1_A2_reference_data.xlsx
@@ -872,12 +872,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>220550</t>
+          <t>220577</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>شيماء شريف محمد عبد الرحمن احمد</t>
+          <t>عبدالرحمن محمد عبداللطيف شهاب</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>220577</t>
+          <t>220615</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>عبدالرحمن محمد عبداللطيف شهاب</t>
+          <t>غاده ابو العلا فتحي ابو العلا ابو الروس</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -926,12 +926,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>220615</t>
+          <t>220616</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>غاده ابو العلا فتحي ابو العلا ابو الروس</t>
+          <t>غاده احمد احمد احمد الشريف</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -953,12 +953,12 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>220616</t>
+          <t>220623</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>غاده احمد احمد احمد الشريف</t>
+          <t>فاطمه احمد محمد محمود كرم</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -980,12 +980,12 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>220623</t>
+          <t>220624</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>فاطمه احمد محمد محمود كرم</t>
+          <t>فاطمه السيد محمد فتحى عطيه الله</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1007,12 +1007,12 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>220624</t>
+          <t>220625</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>فاطمه السيد محمد فتحى عطيه الله</t>
+          <t>فاطمه حموده على عبد الحميد حموده</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1034,12 +1034,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>220625</t>
+          <t>220627</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>فاطمه حموده على عبد الحميد حموده</t>
+          <t>فاطمه عمرو السيد ابراهيم عبد الله</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1061,12 +1061,12 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>220627</t>
+          <t>220628</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>فاطمه عمرو السيد ابراهيم عبد الله</t>
+          <t>فاطمه محمود محمد امام</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1088,12 +1088,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>220628</t>
+          <t>220629</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>فاطمه محمود محمد امام</t>
+          <t>فتحى محمد فتحى السيد عبد الله</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1115,12 +1115,12 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>220629</t>
+          <t>220630</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>فتحى محمد فتحى السيد عبد الله</t>
+          <t>فريده محمود فؤاد محمود</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1142,12 +1142,12 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>220630</t>
+          <t>220635</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>فريده محمود فؤاد محمود</t>
+          <t>كريم ايمن محمد مصطفى ابراهيم</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1169,12 +1169,12 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>220635</t>
+          <t>220636</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>كريم ايمن محمد مصطفى ابراهيم</t>
+          <t>كريم سعيد احمد ابراهيم الحريزى</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1196,12 +1196,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>220636</t>
+          <t>220639</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>كريم سعيد احمد ابراهيم الحريزى</t>
+          <t>كريم مصطفى عبد الرحمن على سعد</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1223,12 +1223,12 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>220639</t>
+          <t>220645</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>كريم مصطفى عبد الرحمن على سعد</t>
+          <t>لجين احمد عبد الله البسطويسى</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1250,12 +1250,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>220645</t>
+          <t>220646</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>لجين احمد عبد الله البسطويسى</t>
+          <t>لجين اشرف جلال عبد الرحمن السمرى</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1277,12 +1277,12 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>220646</t>
+          <t>220647</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>لجين اشرف جلال عبد الرحمن السمرى</t>
+          <t>لوجين السيد محروس اسماعيل</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>A2-A1</t>
+          <t>A2-A2</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1304,12 +1304,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>220647</t>
+          <t>220648</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>لوجين السيد محروس اسماعيل</t>
+          <t>لؤى اكرم عبد الله عبد الفتاح عمر</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1331,12 +1331,12 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>220648</t>
+          <t>220649</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>لؤى اكرم عبد الله عبد الفتاح عمر</t>
+          <t>لؤى على حسين حسن ابو صفيه</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>220649</t>
+          <t>220651</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>لؤى على حسين حسن ابو صفيه</t>
+          <t>ليلى اشرف وصفى</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1385,12 +1385,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>220651</t>
+          <t>220653</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>ليلى اشرف وصفى</t>
+          <t>ماجد حسنى السيد التلاوى</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1412,12 +1412,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>220653</t>
+          <t>220655</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>ماجد حسنى السيد التلاوى</t>
+          <t>مارى مجدى منير عبده</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1439,12 +1439,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>220655</t>
+          <t>220659</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>مارى مجدى منير عبده</t>
+          <t>مالك محمود على محمود زين الدين</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -1466,12 +1466,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>220659</t>
+          <t>220661</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>مالك محمود على محمود زين الدين</t>
+          <t>مبارك السيد إبراهيم بسطويسى جاد الله</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1493,12 +1493,12 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>220661</t>
+          <t>220662</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>مبارك السيد إبراهيم بسطويسى جاد الله</t>
+          <t>مجدى عزوز سعيد عطوه عطيه البنا</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -1520,12 +1520,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>220662</t>
+          <t>220666</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>مجدى عزوز سعيد عطوه عطيه البنا</t>
+          <t>محمد احمد فتحى احمد احمد</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1547,12 +1547,12 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>220666</t>
+          <t>220667</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>محمد احمد فتحى احمد احمد</t>
+          <t>محمد اسامه علاء الدين اللو</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -1574,12 +1574,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>220667</t>
+          <t>220669</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>محمد اسامه علاء الدين اللو</t>
+          <t>محمد السعيد السعيد محمد شعبان</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1601,12 +1601,12 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>220669</t>
+          <t>220670</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>محمد السعيد السعيد محمد شعبان</t>
+          <t>محمد السعيد مسعد مصطفى حراز</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -1628,12 +1628,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>220670</t>
+          <t>220672</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>محمد السعيد مسعد مصطفى حراز</t>
+          <t>محمد الشحات على احمد سرور</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -1655,12 +1655,12 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>220672</t>
+          <t>220673</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>محمد الشحات على احمد سرور</t>
+          <t>محمد أيمن محمد أحمد ناصف</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -1682,12 +1682,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>220673</t>
+          <t>220674</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>محمد أيمن محمد أحمد ناصف</t>
+          <t>محمد باسم عبد الكريم محمود</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -1709,12 +1709,12 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>220674</t>
+          <t>220678</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>محمد باسم عبد الكريم محمود</t>
+          <t>محمد بهاء عبد الحميد عبد الغفار</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -1736,12 +1736,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>220678</t>
+          <t>220679</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>محمد بهاء عبد الحميد عبد الغفار</t>
+          <t>محمد جابر توفيق الشافعى</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1763,12 +1763,12 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>220679</t>
+          <t>220680</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>محمد جابر توفيق الشافعى</t>
+          <t>محمد حسن جلال عبد المجيد وهدان</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -1790,12 +1790,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>220680</t>
+          <t>220683</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>محمد حسن جلال عبد المجيد وهدان</t>
+          <t>محمد سعيد محمود عبد المنعم محمود</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -1817,12 +1817,12 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>220683</t>
+          <t>220684</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>محمد سعيد محمود عبد المنعم محمود</t>
+          <t>محمد صبرى جوده عبد الله خضر</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -1844,12 +1844,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>220684</t>
+          <t>220685</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>محمد صبرى جوده عبد الله خضر</t>
+          <t>محمد صلاح حسن عبد الله حسن</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -1871,12 +1871,12 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>220685</t>
+          <t>220686</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>محمد صلاح حسن عبد الله حسن</t>
+          <t>محمد ضياء الدين محمد شوقى السيد ابراهيم موسى</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -1898,12 +1898,12 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>220686</t>
+          <t>220687</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>محمد ضياء الدين محمد شوقى السيد ابراهيم موسى</t>
+          <t>محمد طارق محمد عبد الرحمن العرينى</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -1925,12 +1925,12 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>220687</t>
+          <t>220688</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>محمد طارق محمد عبد الرحمن العرينى</t>
+          <t>محمد عبد الحفيظ عبد الله محمد على</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -1952,12 +1952,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>220688</t>
+          <t>220689</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>محمد عبد الحفيظ عبد الله محمد على</t>
+          <t>محمد عبد الغفور صبحى عبد الغفور نصير</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -1979,12 +1979,12 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>220689</t>
+          <t>220690</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>محمد عبد الغفور صبحى عبد الغفور نصير</t>
+          <t>محمد عبد النبى عطيه ابو شعيشع</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -2006,12 +2006,12 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>220690</t>
+          <t>220691</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>محمد عبد النبى عطيه ابو شعيشع</t>
+          <t>محمد عبدالهادى عبدالمنعم عمر</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2033,12 +2033,12 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>220691</t>
+          <t>220693</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>محمد عبدالهادى عبدالمنعم عمر</t>
+          <t>محمد علاء محمد عبد العزيز عبد الله</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -2060,12 +2060,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>220693</t>
+          <t>220694</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>محمد علاء محمد عبد العزيز عبد الله</t>
+          <t>محمد على محمد احمد محمد</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2087,12 +2087,12 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>220694</t>
+          <t>220698</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>محمد على محمد احمد محمد</t>
+          <t>محمد محمد احمد الفتيانى</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>A2-A2</t>
+          <t>A2-B1</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>220698</t>
+          <t>220700</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>محمد محمد احمد الفتيانى</t>
+          <t>محمد محمد عبد الله التهامي</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2141,12 +2141,12 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>220700</t>
+          <t>220701</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>محمد محمد عبد الله التهامي</t>
+          <t>محمد محمد عبد الونيس عبد التواب حسن القارب</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -2168,12 +2168,12 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>220701</t>
+          <t>220702</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>محمد محمد عبد الونيس عبد التواب حسن القارب</t>
+          <t>محمد محيى الدين محمد سيد مكاوى</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2195,12 +2195,12 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>220702</t>
+          <t>220703</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>محمد محيى الدين محمد سيد مكاوى</t>
+          <t>محمد مختار شعبان هلالى سليمان</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2222,12 +2222,12 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>220703</t>
+          <t>220705</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>محمد مختار شعبان هلالى سليمان</t>
+          <t>محمد مفرح عبد الباسط عبد الحليم</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2249,12 +2249,12 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>220705</t>
+          <t>220706</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>محمد مفرح عبد الباسط عبد الحليم</t>
+          <t>محمد وائل محمد العيسوى</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -2276,12 +2276,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>220706</t>
+          <t>220707</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>محمد وائل محمد العيسوى</t>
+          <t>محمد وحيد محمد رزق</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2303,12 +2303,12 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>220707</t>
+          <t>220708</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>محمد وحيد محمد رزق</t>
+          <t>محمد ياسر الشافعى محمد على</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -2330,12 +2330,12 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>220708</t>
+          <t>220709</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>محمد ياسر الشافعى محمد على</t>
+          <t>محمد ياسر حامد دياب حمد</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -2357,12 +2357,12 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>220709</t>
+          <t>220710</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>محمد ياسر حامد دياب حمد</t>
+          <t>محمود جمال حسين محمد رسلان</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -2384,12 +2384,12 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>220710</t>
+          <t>220711</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>محمود جمال حسين محمد رسلان</t>
+          <t>مصطفى احمد عبد الخالق عبد العزيز عطعوط</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2411,12 +2411,12 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>220711</t>
+          <t>220712</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>مصطفى احمد عبد الخالق عبد العزيز عطعوط</t>
+          <t>محمود حسن عبد النبى حسين</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -2438,12 +2438,12 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>220712</t>
+          <t>220714</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>محمود حسن عبد النبى حسين</t>
+          <t>محمود كريم شحاته حسن كرد</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -2465,12 +2465,12 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>220714</t>
+          <t>220717</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>محمود كريم شحاته حسن كرد</t>
+          <t>محمود منصور محمود محمد السيد يعقوب</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -2492,12 +2492,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>220717</t>
+          <t>220720</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>محمود منصور محمود محمد السيد يعقوب</t>
+          <t>مروان صبحى ابو الحسن محمد على</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -2519,12 +2519,12 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>220720</t>
+          <t>220721</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>مروان صبحى ابو الحسن محمد على</t>
+          <t>مروان وليد عبدالمنعم عبد القادر ادريس</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -2546,12 +2546,12 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>220721</t>
+          <t>220722</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>مروان وليد عبدالمنعم عبد القادر ادريس</t>
+          <t>مروه عبد الحميد على حسن ايوب</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -2573,12 +2573,12 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>220722</t>
+          <t>220723</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>مروه عبد الحميد على حسن ايوب</t>
+          <t>مريم ابراهيم احمد ابراهيم مبارك</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -2600,12 +2600,12 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>220723</t>
+          <t>220724</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>مريم ابراهيم احمد ابراهيم مبارك</t>
+          <t>مريم الحسن احمد ابراهيم بيومى</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2627,12 +2627,12 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>220724</t>
+          <t>220725</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>مريم الحسن احمد ابراهيم بيومى</t>
+          <t>مريم ايمن عبد الله محمود فخرى</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -2654,12 +2654,12 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>220725</t>
+          <t>220726</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>مريم ايمن عبد الله محمود فخرى</t>
+          <t>مريم ايمن فؤاد عبدالستار</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -2681,12 +2681,12 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>220726</t>
+          <t>220727</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>مريم ايمن فؤاد عبدالستار</t>
+          <t>مريم ايهاب ملاك ثابت</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -2708,12 +2708,12 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>220727</t>
+          <t>220729</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>مريم ايهاب ملاك ثابت</t>
+          <t>مريم رضا محمد ابراهيم صبره</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -2735,12 +2735,12 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>220729</t>
+          <t>220730</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>مريم رضا محمد ابراهيم صبره</t>
+          <t>مريم شعبان مصباح خليفه</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2762,12 +2762,12 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>220730</t>
+          <t>220731</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>مريم شعبان مصباح خليفه</t>
+          <t>مريم شفيق صبحى شفيق حنا</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -2789,12 +2789,12 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>220731</t>
+          <t>220732</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>مريم شفيق صبحى شفيق حنا</t>
+          <t>مريم عمرو يحيى عبده مدنى</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -2816,12 +2816,12 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>220732</t>
+          <t>220733</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>مريم عمرو يحيى عبده مدنى</t>
+          <t>مريم محمد احمد فاروق الديب الشريف</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -2843,12 +2843,12 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>220733</t>
+          <t>220734</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>مريم محمد احمد فاروق الديب الشريف</t>
+          <t>مريم محمد احمد محمد عبد المنعم</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -2870,12 +2870,12 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>220734</t>
+          <t>220735</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>مريم محمد احمد محمد عبد المنعم</t>
+          <t>مريم محمد ثروت صايم مصطفى</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -2897,12 +2897,12 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>220735</t>
+          <t>221051</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>مريم محمد ثروت صايم مصطفى</t>
+          <t>اسراء هشام محمد عبد المنعم</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -2924,12 +2924,12 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>221051</t>
+          <t>220736</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>اسراء هشام محمد عبد المنعم</t>
+          <t>مريم محمد عطيه عبد السلام</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>A2-B1</t>
+          <t>A2-B2</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -2951,12 +2951,12 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>220736</t>
+          <t>220737</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>مريم محمد عطيه عبد السلام</t>
+          <t>مريم محمد محسن عبد الحافظ عبد العظيم</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -2978,12 +2978,12 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>220737</t>
+          <t>220740</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>مريم محمد محسن عبد الحافظ عبد العظيم</t>
+          <t>مصطفى امجد عبد الحليم عبد اللطيف شعبان</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -3005,12 +3005,12 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>220740</t>
+          <t>220742</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>مصطفى امجد عبد الحليم عبد اللطيف شعبان</t>
+          <t>مصطفى عبد الفتاح محمد محمود عبد الفتاح</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -3032,12 +3032,12 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>220742</t>
+          <t>220744</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>مصطفى عبد الفتاح محمد محمود عبد الفتاح</t>
+          <t>مصطفى محمد عبد الله حواش احمد شلبى</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -3059,12 +3059,12 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>220744</t>
+          <t>220745</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>مصطفى محمد عبد الله حواش احمد شلبى</t>
+          <t>مصطفى محمود مصطفى محمود</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -3086,12 +3086,12 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>220745</t>
+          <t>220746</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>مصطفى محمود مصطفى محمود</t>
+          <t>معاذ طاهر محمد شبانه على</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -3113,12 +3113,12 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>220746</t>
+          <t>220747</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>معاذ طاهر محمد شبانه على</t>
+          <t>ملك عبدالغنى احمد حسن</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -3140,12 +3140,12 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>220747</t>
+          <t>220749</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>ملك عبدالغنى احمد حسن</t>
+          <t>ملك ياسر عبد الوهاب محمد الغندور</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -3167,12 +3167,12 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>220749</t>
+          <t>220751</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>ملك ياسر عبد الوهاب محمد الغندور</t>
+          <t>منة الله هانى عبد السميع شكرى</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -3194,12 +3194,12 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>220751</t>
+          <t>220752</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>منة الله هانى عبد السميع شكرى</t>
+          <t>منصور هانى منصور عبدالله</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -3221,12 +3221,12 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>220752</t>
+          <t>220753</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>منصور هانى منصور عبدالله</t>
+          <t>منه الله احمد محمد جمعه عثمان</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -3248,12 +3248,12 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>220753</t>
+          <t>220754</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>منه الله احمد محمد جمعه عثمان</t>
+          <t>منه الله محمد صالح محمد النور</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -3275,12 +3275,12 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>220754</t>
+          <t>220755</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>منه الله محمد صالح محمد النور</t>
+          <t>منه الله محمد عبد الرازق سالم غاليه</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -3302,12 +3302,12 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>220755</t>
+          <t>220756</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>منه الله محمد عبد الرازق سالم غاليه</t>
+          <t>منه عبد الوهاب عبدالله مصطفى</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -3329,12 +3329,12 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>220756</t>
+          <t>220758</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>منه عبد الوهاب عبدالله مصطفى</t>
+          <t>منه محمود محمد احمد</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -3356,12 +3356,12 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>220758</t>
+          <t>220759</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>منه محمود محمد احمد</t>
+          <t>منى عبد الحميد ناصف سيف</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -3383,12 +3383,12 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>220759</t>
+          <t>220760</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>منى عبد الحميد ناصف سيف</t>
+          <t>مهند ابراهيم محمود عبد اللطيف السيد صقر</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -3410,12 +3410,12 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>220760</t>
+          <t>220764</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>مهند ابراهيم محمود عبد اللطيف السيد صقر</t>
+          <t>مياده سلامه قاسم محمد السيد</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -3437,12 +3437,12 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>220764</t>
+          <t>220765</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>مياده سلامه قاسم محمد السيد</t>
+          <t>ميار احمد صبحى السيد السيد</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -3464,12 +3464,12 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>220765</t>
+          <t>220767</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>ميار احمد صبحى السيد السيد</t>
+          <t>ميار صلاح محمد سليمان سليمان</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -3491,12 +3491,12 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>220767</t>
+          <t>220772</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>ميار صلاح محمد سليمان سليمان</t>
+          <t>نجلاء خالد احمد عبد الحميد عبد الواحد</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -3518,12 +3518,12 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>220772</t>
+          <t>220773</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>نجلاء خالد احمد عبد الحميد عبد الواحد</t>
+          <t>ندى اشرف عبد الله ابراهيم</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -3545,12 +3545,12 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>220773</t>
+          <t>220774</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>ندى اشرف عبد الله ابراهيم</t>
+          <t>ندى اشرف محمد محمد</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -3572,12 +3572,12 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>220774</t>
+          <t>220775</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>ندى اشرف محمد محمد</t>
+          <t>ندى حسن السيد احمد عطا الله</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -3599,12 +3599,12 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>220775</t>
+          <t>220776</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>ندى حسن السيد احمد عطا الله</t>
+          <t>ندى عاطف محمد محمد عبده الشيمى</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -3626,12 +3626,12 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>220776</t>
+          <t>220777</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>ندى عاطف محمد محمد عبده الشيمى</t>
+          <t>ندى على زيد عبد الرحمن</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -3653,12 +3653,12 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>220777</t>
+          <t>220778</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>ندى على زيد عبد الرحمن</t>
+          <t>ندى محمد احمد حامد عامر</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -3680,12 +3680,12 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>220778</t>
+          <t>220779</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>ندى محمد احمد حامد عامر</t>
+          <t>نزار عمرو حسن عبد الغنى</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>A2-B2</t>
+          <t>A2-C1</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
@@ -3707,12 +3707,12 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>220779</t>
+          <t>220780</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>نزار عمرو حسن عبد الغنى</t>
+          <t>نصر الدين الابراهيم</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -3734,12 +3734,12 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>220780</t>
+          <t>220781</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>نصر الدين الابراهيم</t>
+          <t>نظمى مصطفى نظمى على عبد النبى</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -3761,12 +3761,12 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>220781</t>
+          <t>220782</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>نظمى مصطفى نظمى على عبد النبى</t>
+          <t>نفيسه محمد محمود عبد الوهاب عبد الفتاح</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
@@ -3788,12 +3788,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>220782</t>
+          <t>220783</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>نفيسه محمد محمود عبد الوهاب عبد الفتاح</t>
+          <t>نهى احمد ابراهيم محمد عيطه</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -3815,12 +3815,12 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>220783</t>
+          <t>220784</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>نهى احمد ابراهيم محمد عيطه</t>
+          <t>نهى على عبد الرحمن على</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -3842,12 +3842,12 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>220784</t>
+          <t>220787</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>نهى على عبد الرحمن على</t>
+          <t>نور محمد عبد الجليل محمد</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -3869,12 +3869,12 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>220787</t>
+          <t>220788</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>نور محمد عبد الجليل محمد</t>
+          <t>نوران اسامه محمد محمود</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
@@ -3896,12 +3896,12 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>220788</t>
+          <t>220789</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>نوران اسامه محمد محمود</t>
+          <t>نوران فوزى شعبان فوزى علام</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -3923,12 +3923,12 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>220789</t>
+          <t>220790</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>نوران فوزى شعبان فوزى علام</t>
+          <t>نورهان حسن عبد الرحمن حسن محمد</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
@@ -3950,12 +3950,12 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>220790</t>
+          <t>220791</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>نورهان حسن عبد الرحمن حسن محمد</t>
+          <t>نورهان محمد عبد العزيز حسن</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -3977,12 +3977,12 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>220791</t>
+          <t>220792</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>نورهان محمد عبد العزيز حسن</t>
+          <t>نورهان محمود السيد محمود اللقانى</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
@@ -4004,12 +4004,12 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>220792</t>
+          <t>220793</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>نورهان محمود السيد محمود اللقانى</t>
+          <t>نورين احمد عبد الحكيم رضوان</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -4031,12 +4031,12 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>220793</t>
+          <t>220794</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>نورين احمد عبد الحكيم رضوان</t>
+          <t>نورين احمد عوده سليمان محمد الشرقاوى</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
@@ -4058,12 +4058,12 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>220794</t>
+          <t>220795</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>نورين احمد عوده سليمان محمد الشرقاوى</t>
+          <t>نيرمين ياسر عبد الجواد احمد عبد الجواد</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -4085,12 +4085,12 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>220795</t>
+          <t>220796</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>نيرمين ياسر عبد الجواد احمد عبد الجواد</t>
+          <t>نيره فوزى فؤاد عبد المنعم ابراهيم</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
@@ -4112,12 +4112,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>220796</t>
+          <t>220797</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>نيره فوزى فؤاد عبد المنعم ابراهيم</t>
+          <t>نيفين احمد سعيد عبد الرحمن الليثى</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>220797</t>
+          <t>220799</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>نيفين احمد سعيد عبد الرحمن الليثى</t>
+          <t>هاجر احمد رمضان سعد الفرحاتى</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -4166,12 +4166,12 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>220799</t>
+          <t>220800</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>هاجر احمد رمضان سعد الفرحاتى</t>
+          <t>هاجر عاطف سيد عبد الجيد احمد</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -4193,12 +4193,12 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>220800</t>
+          <t>220801</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>هاجر عاطف سيد عبد الجيد احمد</t>
+          <t>هايدى محمد حسين رفاعى فراج</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
@@ -4220,12 +4220,12 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>220801</t>
+          <t>220802</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>هايدى محمد حسين رفاعى فراج</t>
+          <t>هدى مدحت خيرى احمد فرج</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -4247,12 +4247,12 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>220802</t>
+          <t>220803</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>هدى مدحت خيرى احمد فرج</t>
+          <t>هرمينا عبد الله جاد جرجس</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
@@ -4274,12 +4274,12 @@
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>220803</t>
+          <t>220804</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>هرمينا عبد الله جاد جرجس</t>
+          <t>هنا خليل عبد الرؤف محمد سعيد</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -4301,12 +4301,12 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>220804</t>
+          <t>220805</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>هنا خليل عبد الرؤف محمد سعيد</t>
+          <t>وسام ايمن على الشريف</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -4328,12 +4328,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>220805</t>
+          <t>220807</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>وسام ايمن على الشريف</t>
+          <t>وليد ياسر عبد الشافى محمود</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -4355,12 +4355,12 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>220807</t>
+          <t>220808</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>وليد ياسر عبد الشافى محمود</t>
+          <t>ياسمين عادل السيد الفرغلى حسن</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
@@ -4382,12 +4382,12 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>220808</t>
+          <t>220809</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>ياسمين عادل السيد الفرغلى حسن</t>
+          <t>يحيى احمد محمد عبد الفتاح الزيات</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -4409,12 +4409,12 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>220809</t>
+          <t>220810</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>يحيى احمد محمد عبد الفتاح الزيات</t>
+          <t>يحيى محمد يحى على</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -4436,12 +4436,12 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>220810</t>
+          <t>220813</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>يحيى محمد يحى على</t>
+          <t>يمنى صلاح عبد الغفار محيسن دسوقى</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -4463,12 +4463,12 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>220813</t>
+          <t>220814</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>يمنى صلاح عبد الغفار محيسن دسوقى</t>
+          <t>يوسف جلال محمد عبد الفتاح صالح</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -4490,12 +4490,12 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>220814</t>
+          <t>220890</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>يوسف جلال محمد عبد الفتاح صالح</t>
+          <t>يوسف حسين ناجي الصرايره</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
@@ -4517,12 +4517,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>220890</t>
+          <t>220815</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>يوسف حسين ناجي الصرايره</t>
+          <t>يوسف حمدى احمد طاجن</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>A2-C1</t>
+          <t>A2-C2</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
@@ -4544,12 +4544,12 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>220815</t>
+          <t>220816</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>يوسف حمدى احمد طاجن</t>
+          <t>يوسف عمرو على حفنى ابراهيم</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
@@ -4571,12 +4571,12 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>220816</t>
+          <t>220817</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>يوسف عمرو على حفنى ابراهيم</t>
+          <t>يوسف فهيم عبد الحميد ابو عزيز</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -4598,12 +4598,12 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>220817</t>
+          <t>220818</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>يوسف فهيم عبد الحميد ابو عزيز</t>
+          <t>يوسف محمد رضا جلال احمد سيد احمد</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -4625,12 +4625,12 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>220818</t>
+          <t>220819</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>يوسف محمد رضا جلال احمد سيد احمد</t>
+          <t>يوسف محمد محمد السيد البطه</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -4652,12 +4652,12 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>220819</t>
+          <t>220820</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>يوسف محمد محمد السيد البطه</t>
+          <t>يوسف محمود محمد ابراهيم</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
@@ -4679,12 +4679,12 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>220820</t>
+          <t>220821</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>يوسف محمود محمد ابراهيم</t>
+          <t>يوسف مصطفى محمد رسلان</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -4706,12 +4706,12 @@
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>220821</t>
+          <t>220822</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>يوسف مصطفى محمد رسلان</t>
+          <t>يوسف مصطفى مصطفى محمد</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -4733,12 +4733,12 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>220822</t>
+          <t>220824</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>يوسف مصطفى مصطفى محمد</t>
+          <t>يوسف وائل حامد ابراهيم العالم</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -4760,12 +4760,12 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>220824</t>
+          <t>220825</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>يوسف وائل حامد ابراهيم العالم</t>
+          <t>يوسف سيد محمد يوسف</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -4787,12 +4787,12 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>220825</t>
+          <t>220826</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>يوسف سيد محمد يوسف</t>
+          <t>عبد الله خالد احمد باحاذق</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
@@ -4814,12 +4814,12 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>220826</t>
+          <t>220827</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>عبد الله خالد احمد باحاذق</t>
+          <t>أبوبكر طارق أبوبكر رمضان</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -4841,12 +4841,12 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>220827</t>
+          <t>220829</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>أبوبكر طارق أبوبكر رمضان</t>
+          <t>تبارك رائد حسن كميل</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
@@ -4868,12 +4868,12 @@
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>220829</t>
+          <t>220830</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>تبارك رائد حسن كميل</t>
+          <t>مصطفى محمد على</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -4895,12 +4895,12 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>220830</t>
+          <t>220832</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>مصطفى محمد على</t>
+          <t>احمد عبد الله نعمان محمد</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -4922,12 +4922,12 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>220832</t>
+          <t>220833</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>احمد عبد الله نعمان محمد</t>
+          <t>رغد فيصل عقيل العمايري</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -4949,12 +4949,12 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>220833</t>
+          <t>220834</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>رغد فيصل عقيل العمايري</t>
+          <t>احمد سليمان محمد</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
@@ -4976,12 +4976,12 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>220834</t>
+          <t>220838</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>احمد سليمان محمد</t>
+          <t>حمزه طارق الطراد</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -5003,12 +5003,12 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>220838</t>
+          <t>220839</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>حمزه طارق الطراد</t>
+          <t>عزام نبيل يحي العمير</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
@@ -5030,12 +5030,12 @@
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>220839</t>
+          <t>220848</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>عزام نبيل يحي العمير</t>
+          <t>عبد الله مسعود مصطفى</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -5057,12 +5057,12 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>220848</t>
+          <t>220853</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>عبد الله مسعود مصطفى</t>
+          <t>قند عدي بدران</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
@@ -5084,12 +5084,12 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>220853</t>
+          <t>220856</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>قند عدي بدران</t>
+          <t>ماسه بلال الدهبي</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -5111,12 +5111,12 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>220856</t>
+          <t>220857</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>ماسه بلال الدهبي</t>
+          <t>محمد عبده علوي محمد</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
@@ -5138,12 +5138,12 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>220857</t>
+          <t>220867</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>محمد عبده علوي محمد</t>
+          <t>شهد جمعه على عبد الفتاح</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -5165,12 +5165,12 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>220867</t>
+          <t>220876</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>شهد جمعه على عبد الفتاح</t>
+          <t>عبد المهيمن مهند سلمان</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
@@ -5192,12 +5192,12 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>220876</t>
+          <t>220878</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>عبد المهيمن مهند سلمان</t>
+          <t>عاصم بن عبد الرحمن بن احمد بامعلم</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -5219,12 +5219,12 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>220878</t>
+          <t>220879</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>عاصم بن عبد الرحمن بن احمد بامعلم</t>
+          <t>علي بن محمد بن على المحمد صالح</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
@@ -5246,12 +5246,12 @@
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>220879</t>
+          <t>221018</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>علي بن محمد بن على المحمد صالح</t>
+          <t>رامي احمد الخطيب</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -5273,12 +5273,12 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>221018</t>
+          <t>221335</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>رامي احمد الخطيب</t>
+          <t>حذيفه طريف القطرنجى</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -5300,12 +5300,12 @@
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>221335</t>
+          <t>220896</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>حذيفه طريف القطرنجى</t>
+          <t>احمد السر ميرغني عمر</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>A2-C2</t>
+          <t>A2-D1</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
@@ -5327,12 +5327,12 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>220896</t>
+          <t>220900</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>احمد السر ميرغني عمر</t>
+          <t>ديما حسن نصر الله الزاملي</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
@@ -5354,12 +5354,12 @@
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>220900</t>
+          <t>220902</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>ديما حسن نصر الله الزاملي</t>
+          <t>كاتيا منيمنة</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
@@ -5381,12 +5381,12 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>220902</t>
+          <t>220908</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>كاتيا منيمنة</t>
+          <t>عمرو زين العابدين طلعت عابدين</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -5408,12 +5408,12 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>220908</t>
+          <t>220909</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>عمرو زين العابدين طلعت عابدين</t>
+          <t>احمد جمال محمد عليمى محمد</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -5435,12 +5435,12 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>220909</t>
+          <t>220912</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>احمد جمال محمد عليمى محمد</t>
+          <t>شيماء بدر زبير علي</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
@@ -5462,12 +5462,12 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>220912</t>
+          <t>220914</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>شيماء بدر زبير علي</t>
+          <t>محمد بن ضيف الله بن رزق الصبحى</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
@@ -5489,12 +5489,12 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>220914</t>
+          <t>220919</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>محمد بن ضيف الله بن رزق الصبحى</t>
+          <t>احمد سليم عيسى ابو لاوى</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
@@ -5516,12 +5516,12 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>220919</t>
+          <t>220920</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>احمد سليم عيسى ابو لاوى</t>
+          <t>دارين محمد طاهر</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -5543,12 +5543,12 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>220920</t>
+          <t>220925</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>دارين محمد طاهر</t>
+          <t>دينا زياد ابراهيم زقماط</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
@@ -5570,12 +5570,12 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>220925</t>
+          <t>220927</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>دينا زياد ابراهيم زقماط</t>
+          <t>سعيد احمد سعيد محمد عبدالسيد</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
@@ -5597,12 +5597,12 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>220927</t>
+          <t>220928</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>سعيد احمد سعيد محمد عبدالسيد</t>
+          <t>ابراهيم عبدالفتاح ابراهيم السروري</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
@@ -5624,12 +5624,12 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>220928</t>
+          <t>220929</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>ابراهيم عبدالفتاح ابراهيم السروري</t>
+          <t>الوليد بن عبدالله بن محمد عامر</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
@@ -5651,12 +5651,12 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>220929</t>
+          <t>220930</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>الوليد بن عبدالله بن محمد عامر</t>
+          <t>يوسف نبيل فريد شاهين</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
@@ -5678,12 +5678,12 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>220930</t>
+          <t>220937</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>يوسف نبيل فريد شاهين</t>
+          <t>اسيل يحيى محمد المزايده</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
@@ -5705,12 +5705,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>220937</t>
+          <t>220940</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>اسيل يحيى محمد المزايده</t>
+          <t>عبدالرحمن محمد محسن الزقري</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -5732,12 +5732,12 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>220940</t>
+          <t>220942</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>عبدالرحمن محمد محسن الزقري</t>
+          <t>عدي علي فلاح الحديد</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
@@ -5759,12 +5759,12 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>220942</t>
+          <t>220947</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>عدي علي فلاح الحديد</t>
+          <t>مهند عبد الفتاح سلام مقبل</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
@@ -5786,12 +5786,12 @@
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
         <is>
-          <t>220947</t>
+          <t>220950</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>مهند عبد الفتاح سلام مقبل</t>
+          <t>يوسف اسماعيل ابراهيم احمد</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
@@ -5813,12 +5813,12 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>220950</t>
+          <t>220951</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>يوسف اسماعيل ابراهيم احمد</t>
+          <t>محمد تيسير محمد ياسين</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
@@ -5840,12 +5840,12 @@
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
         <is>
-          <t>220951</t>
+          <t>220954</t>
         </is>
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>محمد تيسير محمد ياسين</t>
+          <t>طيف فرج علي العماري</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
@@ -5867,12 +5867,12 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>220954</t>
+          <t>220955</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>طيف فرج علي العماري</t>
+          <t>غاده عبدالاله عبدالكريم عبدالله</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
@@ -5894,12 +5894,12 @@
     <row r="202">
       <c r="A202" s="3" t="inlineStr">
         <is>
-          <t>220955</t>
+          <t>220956</t>
         </is>
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>غاده عبدالاله عبدالكريم عبدالله</t>
+          <t>نور الحسين أسعد جاسم العكيلي</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
@@ -5921,12 +5921,12 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>220956</t>
+          <t>220958</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>نور الحسين أسعد جاسم العكيلي</t>
+          <t>محمد حميد حمود علي الديلي</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
@@ -5948,12 +5948,12 @@
     <row r="204">
       <c r="A204" s="3" t="inlineStr">
         <is>
-          <t>220958</t>
+          <t>220959</t>
         </is>
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>محمد حميد حمود علي الديلي</t>
+          <t>ايليا سالم يعقوب المدانات</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
@@ -5975,12 +5975,12 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>220959</t>
+          <t>220961</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>ايليا سالم يعقوب المدانات</t>
+          <t>رهف نزار احمد الامام</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
@@ -6002,12 +6002,12 @@
     <row r="206">
       <c r="A206" s="3" t="inlineStr">
         <is>
-          <t>220961</t>
+          <t>220963</t>
         </is>
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>رهف نزار احمد الامام</t>
+          <t>شهد بنت عبدالله بن حسين ال الصومعي</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
@@ -6029,12 +6029,12 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>220963</t>
+          <t>220964</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>شهد بنت عبدالله بن حسين ال الصومعي</t>
+          <t>ميس غسان مرشد مفارجة</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
@@ -6056,12 +6056,12 @@
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
         <is>
-          <t>220964</t>
+          <t>220966</t>
         </is>
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>ميس غسان مرشد مفارجة</t>
+          <t>عبدالقادر يوسف عبدالقادر ابوسعدة</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
@@ -6083,12 +6083,12 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>220966</t>
+          <t>220762</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>عبدالقادر يوسف عبدالقادر ابوسعدة</t>
+          <t>مؤيد وليد علي كرجه</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>A2-D1</t>
+          <t>A2-D2</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
@@ -6110,12 +6110,12 @@
     <row r="210">
       <c r="A210" s="3" t="inlineStr">
         <is>
-          <t>220762</t>
+          <t>220845</t>
         </is>
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>مؤيد وليد علي كرجه</t>
+          <t>ريان تاج الدين عبد الله أحمد</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
@@ -6137,12 +6137,12 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>220845</t>
+          <t>220889</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>ريان تاج الدين عبد الله أحمد</t>
+          <t>سجى السر ميرغني عمر</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
@@ -6164,12 +6164,12 @@
     <row r="212">
       <c r="A212" s="3" t="inlineStr">
         <is>
-          <t>220889</t>
+          <t>220969</t>
         </is>
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>سجى السر ميرغني عمر</t>
+          <t>نهال حسام زهره</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
@@ -6191,12 +6191,12 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>220969</t>
+          <t>220970</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>نهال حسام زهره</t>
+          <t>مبارك حسن ابراهيم</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
@@ -6218,12 +6218,12 @@
     <row r="214">
       <c r="A214" s="3" t="inlineStr">
         <is>
-          <t>220970</t>
+          <t>220971</t>
         </is>
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>مبارك حسن ابراهيم</t>
+          <t>فراس حسين نعيم الكوز</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
@@ -6245,12 +6245,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>220971</t>
+          <t>220972</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>فراس حسين نعيم الكوز</t>
+          <t>عاصم عبدالحكيم محمد سعيد ناصر</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -6272,12 +6272,12 @@
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
         <is>
-          <t>220972</t>
+          <t>220974</t>
         </is>
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>عاصم عبدالحكيم محمد سعيد ناصر</t>
+          <t>مايا رضوان احمد سالم</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
@@ -6299,12 +6299,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>220974</t>
+          <t>220979</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>مايا رضوان احمد سالم</t>
+          <t>محمد حسين محمد الحامد</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -6326,12 +6326,12 @@
     <row r="218">
       <c r="A218" s="3" t="inlineStr">
         <is>
-          <t>220979</t>
+          <t>220983</t>
         </is>
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>محمد حسين محمد الحامد</t>
+          <t>حسام محمد احمد الكوز</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
@@ -6353,12 +6353,12 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>220983</t>
+          <t>220986</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>حسام محمد احمد الكوز</t>
+          <t>هاشم احمد صالح الشرجي</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
@@ -6380,12 +6380,12 @@
     <row r="220">
       <c r="A220" s="3" t="inlineStr">
         <is>
-          <t>220986</t>
+          <t>220989</t>
         </is>
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>هاشم احمد صالح الشرجي</t>
+          <t>مشاري محمد يحيي الكحلاني</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
@@ -6407,12 +6407,12 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>220989</t>
+          <t>220991</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>مشاري محمد يحيي الكحلاني</t>
+          <t>عمر حسام الدين الزيبق</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
@@ -6434,12 +6434,12 @@
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
         <is>
-          <t>220991</t>
+          <t>220992</t>
         </is>
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>عمر حسام الدين الزيبق</t>
+          <t>يحيى عبدالغني بني</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
@@ -6461,12 +6461,12 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>220992</t>
+          <t>220996</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>يحيى عبدالغني بني</t>
+          <t>صفية وفائي</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
@@ -6488,12 +6488,12 @@
     <row r="224">
       <c r="A224" s="3" t="inlineStr">
         <is>
-          <t>220996</t>
+          <t>220997</t>
         </is>
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>صفية وفائي</t>
+          <t>احمد عماد الدين محمد عبد الرحمن</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
@@ -6515,12 +6515,12 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>220997</t>
+          <t>221002</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>احمد عماد الدين محمد عبد الرحمن</t>
+          <t>هاجر مؤيد السلوم</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
@@ -6542,12 +6542,12 @@
     <row r="226">
       <c r="A226" s="3" t="inlineStr">
         <is>
-          <t>221002</t>
+          <t>221006</t>
         </is>
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>هاجر مؤيد السلوم</t>
+          <t>فهد هارون ادم محمد</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
@@ -6569,12 +6569,12 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>221006</t>
+          <t>221008</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>فهد هارون ادم محمد</t>
+          <t>وفاق عبدالوهاب محمد ابراهيم</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
@@ -6596,12 +6596,12 @@
     <row r="228">
       <c r="A228" s="3" t="inlineStr">
         <is>
-          <t>221008</t>
+          <t>221012</t>
         </is>
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>وفاق عبدالوهاب محمد ابراهيم</t>
+          <t>اسامه الشيخ احمد الامام</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
@@ -6623,12 +6623,12 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>221012</t>
+          <t>221015</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>اسامه الشيخ احمد الامام</t>
+          <t>وفاء حسين ميرغنى محمود</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
@@ -6650,12 +6650,12 @@
     <row r="230">
       <c r="A230" s="3" t="inlineStr">
         <is>
-          <t>221015</t>
+          <t>221016</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>وفاء حسين ميرغنى محمود</t>
+          <t>ايمن ناصر محمد ابو ديه</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
@@ -6677,12 +6677,12 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>221016</t>
+          <t>221020</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>ايمن ناصر محمد ابو ديه</t>
+          <t>مي سلوم سالم لم يصعد</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -6704,12 +6704,12 @@
     <row r="232">
       <c r="A232" s="3" t="inlineStr">
         <is>
-          <t>221020</t>
+          <t>221021</t>
         </is>
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>مي سلوم سالم لم يصعد</t>
+          <t>عثمان ابوالقاسم احمد حسن</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
@@ -6731,12 +6731,12 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>221021</t>
+          <t>221023</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>عثمان ابوالقاسم احمد حسن</t>
+          <t>مرام عبدالله محمد حامد</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -6758,12 +6758,12 @@
     <row r="234">
       <c r="A234" s="3" t="inlineStr">
         <is>
-          <t>221023</t>
+          <t>221025</t>
         </is>
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>مرام عبدالله محمد حامد</t>
+          <t>بتول محمد يوسف</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
@@ -6785,12 +6785,12 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>221025</t>
+          <t>221029</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>بتول محمد يوسف</t>
+          <t>معتصم توفيق محمد بكرون</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
@@ -6812,12 +6812,12 @@
     <row r="236">
       <c r="A236" s="3" t="inlineStr">
         <is>
-          <t>221029</t>
+          <t>221035</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>معتصم توفيق محمد بكرون</t>
+          <t>محمد بدر احمد علي مول الدويله</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
@@ -6839,12 +6839,12 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>221035</t>
+          <t>221036</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>محمد بدر احمد علي مول الدويله</t>
+          <t>عبد السلام وليد عبد السلام ابو حلوان</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
@@ -6866,12 +6866,12 @@
     <row r="238">
       <c r="A238" s="3" t="inlineStr">
         <is>
-          <t>221036</t>
+          <t>221037</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>عبد السلام وليد عبد السلام ابو حلوان</t>
+          <t>رنا بنت عبد الغني بن بكر برناوي</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
@@ -6893,12 +6893,12 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>221037</t>
+          <t>221040</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>رنا بنت عبد الغني بن بكر برناوي</t>
+          <t>محمد الطاهر محمد الطاهر</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
@@ -6920,12 +6920,12 @@
     <row r="240">
       <c r="A240" s="3" t="inlineStr">
         <is>
-          <t>221040</t>
+          <t>221046</t>
         </is>
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>محمد الطاهر محمد الطاهر</t>
+          <t>احمد مجدي امين محمد</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
@@ -6947,12 +6947,12 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>221046</t>
+          <t>221047</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>احمد مجدي امين محمد</t>
+          <t>احمد محسن محمد ماهر ابو هاشم</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>A2-D2</t>
+          <t>A2-E1</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
@@ -6974,12 +6974,12 @@
     <row r="242">
       <c r="A242" s="3" t="inlineStr">
         <is>
-          <t>221047</t>
+          <t>221048</t>
         </is>
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>احمد محسن محمد ماهر ابو هاشم</t>
+          <t>احمد محمد اسامة احمد عبدالخالق احمد</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
@@ -7001,12 +7001,12 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>221048</t>
+          <t>221049</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>احمد محمد اسامة احمد عبدالخالق احمد</t>
+          <t>ادهم عامر عبدالحافظ احمد محمد</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr">
@@ -7028,12 +7028,12 @@
     <row r="244">
       <c r="A244" s="3" t="inlineStr">
         <is>
-          <t>221049</t>
+          <t>221050</t>
         </is>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>ادهم عامر عبدالحافظ احمد محمد</t>
+          <t>اسراء احمد محمد عبد الصادق نور</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
@@ -7055,12 +7055,12 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>221050</t>
+          <t>221052</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>اسراء احمد محمد عبد الصادق نور</t>
+          <t>امنيه سلامه عبده محمد</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
@@ -7082,12 +7082,12 @@
     <row r="246">
       <c r="A246" s="3" t="inlineStr">
         <is>
-          <t>221052</t>
+          <t>221053</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>امنيه سلامه عبده محمد</t>
+          <t>امينه خالد عوض عفيفى تاج الدين</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>221053</t>
+          <t>221054</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>امينه خالد عوض عفيفى تاج الدين</t>
+          <t>انجي علاء سعد الدين الشحات السيد</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
@@ -7136,12 +7136,12 @@
     <row r="248">
       <c r="A248" s="3" t="inlineStr">
         <is>
-          <t>221054</t>
+          <t>221055</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>انجي علاء سعد الدين الشحات السيد</t>
+          <t>ايلاري هاني سند ماضي</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
@@ -7163,12 +7163,12 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>221055</t>
+          <t>221056</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>ايلاري هاني سند ماضي</t>
+          <t>إيريني وجدي عزمي عبدالمسيح</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
@@ -7190,12 +7190,12 @@
     <row r="250">
       <c r="A250" s="3" t="inlineStr">
         <is>
-          <t>221056</t>
+          <t>221059</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>إيريني وجدي عزمي عبدالمسيح</t>
+          <t>أحمد عزت مختار عزت</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
@@ -7217,12 +7217,12 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>221059</t>
+          <t>221060</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>أحمد عزت مختار عزت</t>
+          <t>أحمد مصطفى السيد سالم عبد الرحيم</t>
         </is>
       </c>
       <c r="C251" s="4" t="inlineStr">
@@ -7244,12 +7244,12 @@
     <row r="252">
       <c r="A252" s="3" t="inlineStr">
         <is>
-          <t>221060</t>
+          <t>221062</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>أحمد مصطفى السيد سالم عبد الرحيم</t>
+          <t>أسراء محمد هانى محمد رشدى خليل غفيفى</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>221062</t>
+          <t>221063</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>أسراء محمد هانى محمد رشدى خليل غفيفى</t>
+          <t>أسماء أحمد عبدالله عبد المقصود أحمد</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
@@ -7298,12 +7298,12 @@
     <row r="254">
       <c r="A254" s="3" t="inlineStr">
         <is>
-          <t>221063</t>
+          <t>221064</t>
         </is>
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>أسماء أحمد عبدالله عبد المقصود أحمد</t>
+          <t>أكرم مصطفي فتحي محمد</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
@@ -7325,12 +7325,12 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>221064</t>
+          <t>221066</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>أكرم مصطفي فتحي محمد</t>
+          <t>أية عبدالسميع محمد سليمان</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
@@ -7352,12 +7352,12 @@
     <row r="256">
       <c r="A256" s="3" t="inlineStr">
         <is>
-          <t>221066</t>
+          <t>221067</t>
         </is>
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>أية عبدالسميع محمد سليمان</t>
+          <t>آيتن أحمد مصطفى محمد مصطفى</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
@@ -7379,12 +7379,12 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>221067</t>
+          <t>221068</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>آيتن أحمد مصطفى محمد مصطفى</t>
+          <t>آيه حسن محمد مأمون</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr">
@@ -7406,12 +7406,12 @@
     <row r="258">
       <c r="A258" s="3" t="inlineStr">
         <is>
-          <t>221068</t>
+          <t>221069</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>آيه حسن محمد مأمون</t>
+          <t>بثينه خالد ابراهيم محمد موسى</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
@@ -7433,12 +7433,12 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>221069</t>
+          <t>221070</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>بثينه خالد ابراهيم محمد موسى</t>
+          <t>بسمة علاء حسني زهران</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
@@ -7460,12 +7460,12 @@
     <row r="260">
       <c r="A260" s="3" t="inlineStr">
         <is>
-          <t>221070</t>
+          <t>221071</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>بسمة علاء حسني زهران</t>
+          <t>بسملة وسام صلاح أحمد</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
@@ -7487,12 +7487,12 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>221071</t>
+          <t>221072</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>بسملة وسام صلاح أحمد</t>
+          <t>بسنت احمد شكرالله عبدالباسط</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
@@ -7514,12 +7514,12 @@
     <row r="262">
       <c r="A262" s="3" t="inlineStr">
         <is>
-          <t>221072</t>
+          <t>221073</t>
         </is>
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>بسنت احمد شكرالله عبدالباسط</t>
+          <t>بلال لبيب يسري عبد اللطيف عبد الغني</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
@@ -7541,12 +7541,12 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>221073</t>
+          <t>221075</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>بلال لبيب يسري عبد اللطيف عبد الغني</t>
+          <t>تسنيم اسامة يوسف نعيم</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
@@ -7568,12 +7568,12 @@
     <row r="264">
       <c r="A264" s="3" t="inlineStr">
         <is>
-          <t>221075</t>
+          <t>221076</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>تسنيم اسامة يوسف نعيم</t>
+          <t>تسنيم علاء ناجي عبدالراضي</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
@@ -7595,12 +7595,12 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>221076</t>
+          <t>221077</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>تسنيم علاء ناجي عبدالراضي</t>
+          <t>تقي محمود احمد السمكري</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
@@ -7622,12 +7622,12 @@
     <row r="266">
       <c r="A266" s="3" t="inlineStr">
         <is>
-          <t>221077</t>
+          <t>221078</t>
         </is>
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>تقي محمود احمد السمكري</t>
+          <t>توماس نبيل سامي غطاس</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
@@ -7649,12 +7649,12 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>221078</t>
+          <t>221079</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>توماس نبيل سامي غطاس</t>
+          <t>جنا هاني احمد عبد القادر</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
@@ -7676,12 +7676,12 @@
     <row r="268">
       <c r="A268" s="3" t="inlineStr">
         <is>
-          <t>221079</t>
+          <t>221080</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>جنا هاني احمد عبد القادر</t>
+          <t>جنة الله علاء الدين أحمد عيد</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
@@ -7703,12 +7703,12 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>221080</t>
+          <t>221084</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>جنة الله علاء الدين أحمد عيد</t>
+          <t>جودي احمد السيد سليمان</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
@@ -7730,12 +7730,12 @@
     <row r="270">
       <c r="A270" s="3" t="inlineStr">
         <is>
-          <t>221084</t>
+          <t>220748</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>جودي احمد السيد سليمان</t>
+          <t>ملك عمرو على حسن</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>A2-E1</t>
+          <t>A2-E2</t>
         </is>
       </c>
       <c r="E270" s="3" t="inlineStr">
@@ -7757,12 +7757,12 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>220748</t>
+          <t>221085</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>ملك عمرو على حسن</t>
+          <t>جوفانا روماني راشد شنوده</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
@@ -7784,12 +7784,12 @@
     <row r="272">
       <c r="A272" s="3" t="inlineStr">
         <is>
-          <t>221085</t>
+          <t>221086</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>جوفانا روماني راشد شنوده</t>
+          <t>جونسي صلاح اسماعيل حجازي</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
@@ -7811,12 +7811,12 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>221086</t>
+          <t>221087</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>جونسي صلاح اسماعيل حجازي</t>
+          <t>جونى سامر صفوت فهمى ميخائيل</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
@@ -7838,12 +7838,12 @@
     <row r="274">
       <c r="A274" s="3" t="inlineStr">
         <is>
-          <t>221087</t>
+          <t>221088</t>
         </is>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>جونى سامر صفوت فهمى ميخائيل</t>
+          <t>حبيبة اسماعيل محمد سعيد اسماعيل محرم</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
@@ -7865,12 +7865,12 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>221088</t>
+          <t>221089</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>حبيبة اسماعيل محمد سعيد اسماعيل محرم</t>
+          <t>حبيبة زكي محمد زكي</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr">
@@ -7892,12 +7892,12 @@
     <row r="276">
       <c r="A276" s="3" t="inlineStr">
         <is>
-          <t>221089</t>
+          <t>221090</t>
         </is>
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>حبيبة زكي محمد زكي</t>
+          <t>حبيبه محمد صابر عبدالعال</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
@@ -7919,12 +7919,12 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>221090</t>
+          <t>221091</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>حبيبه محمد صابر عبدالعال</t>
+          <t>حسن احمد حسن الصفتي</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
@@ -7946,12 +7946,12 @@
     <row r="278">
       <c r="A278" s="3" t="inlineStr">
         <is>
-          <t>221091</t>
+          <t>221092</t>
         </is>
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>حسن احمد حسن الصفتي</t>
+          <t>حسن محمد حسن شمس الدين</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
@@ -7973,12 +7973,12 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>221092</t>
+          <t>221093</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>حسن محمد حسن شمس الدين</t>
+          <t>حلا احمد محمد محمد فضل الله</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
@@ -8000,12 +8000,12 @@
     <row r="280">
       <c r="A280" s="3" t="inlineStr">
         <is>
-          <t>221093</t>
+          <t>221095</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>حلا احمد محمد محمد فضل الله</t>
+          <t>حمزه هشام بكر ابو القميز</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
@@ -8027,12 +8027,12 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>221095</t>
+          <t>221096</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>حمزه هشام بكر ابو القميز</t>
+          <t>حنين طارق محرم شلبي</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -8054,12 +8054,12 @@
     <row r="282">
       <c r="A282" s="3" t="inlineStr">
         <is>
-          <t>221096</t>
+          <t>221097</t>
         </is>
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>حنين طارق محرم شلبي</t>
+          <t>خالد علاء عبد السميع عبدالله الديب</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
@@ -8081,12 +8081,12 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>221097</t>
+          <t>221099</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>خالد علاء عبد السميع عبدالله الديب</t>
+          <t>دارين أحمد فرج القاصد</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
@@ -8108,12 +8108,12 @@
     <row r="284">
       <c r="A284" s="3" t="inlineStr">
         <is>
-          <t>221099</t>
+          <t>221100</t>
         </is>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>دارين أحمد فرج القاصد</t>
+          <t>دارين السيد مصيلحي مصيلحي</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
@@ -8135,12 +8135,12 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>221100</t>
+          <t>221101</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>دارين السيد مصيلحي مصيلحي</t>
+          <t>دارين محمد ابراهيم ماضى</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
@@ -8162,12 +8162,12 @@
     <row r="286">
       <c r="A286" s="3" t="inlineStr">
         <is>
-          <t>221101</t>
+          <t>221102</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>دارين محمد ابراهيم ماضى</t>
+          <t>دانا أسامة عبدالغني محمد</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
@@ -8189,12 +8189,12 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>221102</t>
+          <t>221103</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>دانا أسامة عبدالغني محمد</t>
+          <t>دانه عبداللطيف فؤاد زيان</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
@@ -8216,12 +8216,12 @@
     <row r="288">
       <c r="A288" s="3" t="inlineStr">
         <is>
-          <t>221103</t>
+          <t>221104</t>
         </is>
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>دانه عبداللطيف فؤاد زيان</t>
+          <t>دعاء أشرف أحمد عبد الله</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
@@ -8243,12 +8243,12 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>221104</t>
+          <t>221106</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>دعاء أشرف أحمد عبد الله</t>
+          <t>دينا ناجي عبد المنعم الشيخ</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
@@ -8270,12 +8270,12 @@
     <row r="290">
       <c r="A290" s="3" t="inlineStr">
         <is>
-          <t>221106</t>
+          <t>221108</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>دينا ناجي عبد المنعم الشيخ</t>
+          <t>رانيا عادل طلخان رزق</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
@@ -8297,12 +8297,12 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>221108</t>
+          <t>221110</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>رانيا عادل طلخان رزق</t>
+          <t>رفيده أيمن مصطفى النحاس شحاته</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
@@ -8324,12 +8324,12 @@
     <row r="292">
       <c r="A292" s="3" t="inlineStr">
         <is>
-          <t>221110</t>
+          <t>221111</t>
         </is>
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>رفيده أيمن مصطفى النحاس شحاته</t>
+          <t>رنا عمرو محمد شرايحي</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
@@ -8351,12 +8351,12 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>221111</t>
+          <t>221112</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>رنا عمرو محمد شرايحي</t>
+          <t>رنيم ايمن علي علام</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
@@ -8378,12 +8378,12 @@
     <row r="294">
       <c r="A294" s="3" t="inlineStr">
         <is>
-          <t>221112</t>
+          <t>221114</t>
         </is>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>رنيم ايمن علي علام</t>
+          <t>روان محمد ياسر عبد العال ابو الوفا</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
@@ -8405,12 +8405,12 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>221114</t>
+          <t>221116</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>روان محمد ياسر عبد العال ابو الوفا</t>
+          <t>روينا محمد عبدالحكيم الاشموني</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
@@ -8432,12 +8432,12 @@
     <row r="296">
       <c r="A296" s="3" t="inlineStr">
         <is>
-          <t>221116</t>
+          <t>221117</t>
         </is>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>روينا محمد عبدالحكيم الاشموني</t>
+          <t>رؤى طارق مرسى محمود</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
@@ -8459,12 +8459,12 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>221117</t>
+          <t>221118</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>رؤى طارق مرسى محمود</t>
+          <t>ريم السيد صالح خليل</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
@@ -8486,12 +8486,12 @@
     <row r="298">
       <c r="A298" s="3" t="inlineStr">
         <is>
-          <t>221118</t>
+          <t>221119</t>
         </is>
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>ريم السيد صالح خليل</t>
+          <t>زياد شريف حلمي الألفي</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
@@ -8513,12 +8513,12 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>221119</t>
+          <t>221120</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>زياد شريف حلمي الألفي</t>
+          <t>سارة علاءالدين احمد محمد</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
@@ -8540,12 +8540,12 @@
     <row r="300">
       <c r="A300" s="3" t="inlineStr">
         <is>
-          <t>221120</t>
+          <t>221121</t>
         </is>
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>سارة علاءالدين احمد محمد</t>
+          <t>سارة احمد محمد على خليل</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
@@ -8567,12 +8567,12 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>221121</t>
+          <t>220449</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>سارة احمد محمد على خليل</t>
+          <t>حبيبة الله وائل البرماوى</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>A2-E2</t>
+          <t>A2-F1</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
@@ -8594,12 +8594,12 @@
     <row r="302">
       <c r="A302" s="3" t="inlineStr">
         <is>
-          <t>220449</t>
+          <t>220550</t>
         </is>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>حبيبة الله وائل البرماوى</t>
+          <t>شيماء شريف محمد عبد الرحمن احمد</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">

</xml_diff>